<commit_message>
Trend: re-anchor charts on a wider grid so the two columns no longer overlap
</commit_message>
<xml_diff>
--- a/output/Competitor_Scorecard.xlsx
+++ b/output/Competitor_Scorecard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Claude_Projects\competitor-scorecard\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E74495F4-DAA7-46E1-BB6C-0F275F60E4D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD388868-6952-4749-8DD6-EDC62432437B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2374,7 +2374,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$68</c:f>
+              <c:f>Trend!$A$76</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2395,7 +2395,7 @@
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -2433,7 +2433,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$68:$K$68</c:f>
+              <c:f>Trend!$B$76:$K$76</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2485,7 +2485,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C5FC-4A26-B1C5-C71B6498DBED}"/>
+              <c16:uniqueId val="{00000000-77F7-466E-810F-3AE1E211D6AD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2498,8 +2498,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="64986800"/>
-        <c:axId val="2115073552"/>
+        <c:axId val="1206437903"/>
+        <c:axId val="1142377711"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2509,7 +2509,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$63</c:f>
+              <c:f>Trend!$A$71</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2543,7 +2543,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -2581,7 +2581,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$63:$K$63</c:f>
+              <c:f>Trend!$B$71:$K$71</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2621,7 +2621,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-C5FC-4A26-B1C5-C71B6498DBED}"/>
+              <c16:uniqueId val="{00000001-77F7-466E-810F-3AE1E211D6AD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2630,7 +2630,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$64</c:f>
+              <c:f>Trend!$A$72</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2664,7 +2664,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -2702,7 +2702,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$64:$K$64</c:f>
+              <c:f>Trend!$B$72:$K$72</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2742,7 +2742,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-C5FC-4A26-B1C5-C71B6498DBED}"/>
+              <c16:uniqueId val="{00000002-77F7-466E-810F-3AE1E211D6AD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2751,7 +2751,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$65</c:f>
+              <c:f>Trend!$A$73</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2785,7 +2785,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -2823,7 +2823,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$65:$K$65</c:f>
+              <c:f>Trend!$B$73:$K$73</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2863,7 +2863,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-C5FC-4A26-B1C5-C71B6498DBED}"/>
+              <c16:uniqueId val="{00000003-77F7-466E-810F-3AE1E211D6AD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2872,7 +2872,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$66</c:f>
+              <c:f>Trend!$A$74</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2906,7 +2906,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -2944,7 +2944,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$66:$K$66</c:f>
+              <c:f>Trend!$B$74:$K$74</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2984,7 +2984,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-C5FC-4A26-B1C5-C71B6498DBED}"/>
+              <c16:uniqueId val="{00000004-77F7-466E-810F-3AE1E211D6AD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2993,7 +2993,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$67</c:f>
+              <c:f>Trend!$A$75</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3027,7 +3027,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -3065,7 +3065,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$67:$K$67</c:f>
+              <c:f>Trend!$B$75:$K$75</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3105,7 +3105,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-C5FC-4A26-B1C5-C71B6498DBED}"/>
+              <c16:uniqueId val="{00000005-77F7-466E-810F-3AE1E211D6AD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3182,7 +3182,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="2115073552"/>
+        <c:axId val="1142377711"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -3217,12 +3217,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="64986800"/>
+        <c:crossAx val="1206437903"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="64986800"/>
+        <c:axId val="1206437903"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3232,7 +3232,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="2115073552"/>
+        <c:crossAx val="1142377711"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -3291,7 +3291,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$74</c:f>
+              <c:f>Trend!$A$82</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3312,7 +3312,7 @@
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -3350,7 +3350,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$74:$K$74</c:f>
+              <c:f>Trend!$B$82:$K$82</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3402,7 +3402,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-23F6-447A-BD00-5A7D0487E809}"/>
+              <c16:uniqueId val="{00000000-BF57-4996-9771-C80C6FD48ABC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3415,8 +3415,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="64993760"/>
-        <c:axId val="2115073072"/>
+        <c:axId val="1658447375"/>
+        <c:axId val="1142400271"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -3426,7 +3426,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$70</c:f>
+              <c:f>Trend!$A$78</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3460,7 +3460,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -3498,7 +3498,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$70:$K$70</c:f>
+              <c:f>Trend!$B$78:$K$78</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3538,7 +3538,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-23F6-447A-BD00-5A7D0487E809}"/>
+              <c16:uniqueId val="{00000001-BF57-4996-9771-C80C6FD48ABC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3547,7 +3547,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$71</c:f>
+              <c:f>Trend!$A$79</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3581,7 +3581,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -3619,7 +3619,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$71:$K$71</c:f>
+              <c:f>Trend!$B$79:$K$79</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3659,7 +3659,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-23F6-447A-BD00-5A7D0487E809}"/>
+              <c16:uniqueId val="{00000002-BF57-4996-9771-C80C6FD48ABC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3668,7 +3668,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$72</c:f>
+              <c:f>Trend!$A$80</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3702,7 +3702,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -3740,7 +3740,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$72:$K$72</c:f>
+              <c:f>Trend!$B$80:$K$80</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3780,7 +3780,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-23F6-447A-BD00-5A7D0487E809}"/>
+              <c16:uniqueId val="{00000003-BF57-4996-9771-C80C6FD48ABC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3789,7 +3789,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$73</c:f>
+              <c:f>Trend!$A$81</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3823,7 +3823,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -3861,7 +3861,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$73:$K$73</c:f>
+              <c:f>Trend!$B$81:$K$81</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3901,7 +3901,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-23F6-447A-BD00-5A7D0487E809}"/>
+              <c16:uniqueId val="{00000004-BF57-4996-9771-C80C6FD48ABC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3978,7 +3978,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="2115073072"/>
+        <c:axId val="1142400271"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4013,12 +4013,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="64993760"/>
+        <c:crossAx val="1658447375"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="64993760"/>
+        <c:axId val="1658447375"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4028,7 +4028,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="2115073072"/>
+        <c:crossAx val="1142400271"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -4087,7 +4087,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$81</c:f>
+              <c:f>Trend!$A$89</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4108,7 +4108,7 @@
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -4146,7 +4146,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$81:$K$81</c:f>
+              <c:f>Trend!$B$89:$K$89</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -4198,7 +4198,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C344-4EC0-8710-C5DB66EC9F97}"/>
+              <c16:uniqueId val="{00000000-3652-4AEE-84BD-917EB6877A71}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4211,8 +4211,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="64978448"/>
-        <c:axId val="2115088912"/>
+        <c:axId val="1658447839"/>
+        <c:axId val="1142392111"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -4222,7 +4222,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$76</c:f>
+              <c:f>Trend!$A$84</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4256,7 +4256,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -4294,7 +4294,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$76:$K$76</c:f>
+              <c:f>Trend!$B$84:$K$84</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -4334,7 +4334,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-C344-4EC0-8710-C5DB66EC9F97}"/>
+              <c16:uniqueId val="{00000001-3652-4AEE-84BD-917EB6877A71}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4343,7 +4343,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$77</c:f>
+              <c:f>Trend!$A$85</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4377,7 +4377,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -4415,7 +4415,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$77:$K$77</c:f>
+              <c:f>Trend!$B$85:$K$85</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -4455,7 +4455,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-C344-4EC0-8710-C5DB66EC9F97}"/>
+              <c16:uniqueId val="{00000002-3652-4AEE-84BD-917EB6877A71}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4464,7 +4464,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$78</c:f>
+              <c:f>Trend!$A$86</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4498,7 +4498,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -4536,7 +4536,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$78:$K$78</c:f>
+              <c:f>Trend!$B$86:$K$86</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -4576,7 +4576,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-C344-4EC0-8710-C5DB66EC9F97}"/>
+              <c16:uniqueId val="{00000003-3652-4AEE-84BD-917EB6877A71}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4585,7 +4585,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$79</c:f>
+              <c:f>Trend!$A$87</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4619,7 +4619,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -4657,7 +4657,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$79:$K$79</c:f>
+              <c:f>Trend!$B$87:$K$87</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -4697,7 +4697,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-C344-4EC0-8710-C5DB66EC9F97}"/>
+              <c16:uniqueId val="{00000004-3652-4AEE-84BD-917EB6877A71}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4706,7 +4706,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$80</c:f>
+              <c:f>Trend!$A$88</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4740,7 +4740,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -4778,7 +4778,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$80:$K$80</c:f>
+              <c:f>Trend!$B$88:$K$88</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -4818,7 +4818,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-C344-4EC0-8710-C5DB66EC9F97}"/>
+              <c16:uniqueId val="{00000005-3652-4AEE-84BD-917EB6877A71}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4895,7 +4895,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="2115088912"/>
+        <c:axId val="1142392111"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4930,12 +4930,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="64978448"/>
+        <c:crossAx val="1658447839"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="64978448"/>
+        <c:axId val="1658447839"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4945,7 +4945,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="2115088912"/>
+        <c:crossAx val="1142392111"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -5004,7 +5004,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$87</c:f>
+              <c:f>Trend!$A$95</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5025,7 +5025,7 @@
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -5063,7 +5063,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$87:$K$87</c:f>
+              <c:f>Trend!$B$95:$K$95</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -5115,7 +5115,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1FCD-4D7C-9E44-342BA75DE8D2}"/>
+              <c16:uniqueId val="{00000000-8E9B-40F0-9C5A-A1C094762365}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5128,8 +5128,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="64994688"/>
-        <c:axId val="2115092272"/>
+        <c:axId val="1658445983"/>
+        <c:axId val="1142395951"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -5139,7 +5139,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$83</c:f>
+              <c:f>Trend!$A$91</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5173,7 +5173,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -5211,7 +5211,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$83:$K$83</c:f>
+              <c:f>Trend!$B$91:$K$91</c:f>
               <c:numCache>
                 <c:formatCode>0.00"x"</c:formatCode>
                 <c:ptCount val="10"/>
@@ -5251,7 +5251,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-1FCD-4D7C-9E44-342BA75DE8D2}"/>
+              <c16:uniqueId val="{00000001-8E9B-40F0-9C5A-A1C094762365}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5260,7 +5260,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$84</c:f>
+              <c:f>Trend!$A$92</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5294,7 +5294,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -5332,7 +5332,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$84:$K$84</c:f>
+              <c:f>Trend!$B$92:$K$92</c:f>
               <c:numCache>
                 <c:formatCode>0.00"x"</c:formatCode>
                 <c:ptCount val="10"/>
@@ -5372,7 +5372,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-1FCD-4D7C-9E44-342BA75DE8D2}"/>
+              <c16:uniqueId val="{00000002-8E9B-40F0-9C5A-A1C094762365}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5381,7 +5381,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$85</c:f>
+              <c:f>Trend!$A$93</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5415,7 +5415,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -5453,7 +5453,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$85:$K$85</c:f>
+              <c:f>Trend!$B$93:$K$93</c:f>
               <c:numCache>
                 <c:formatCode>0.00"x"</c:formatCode>
                 <c:ptCount val="10"/>
@@ -5493,7 +5493,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-1FCD-4D7C-9E44-342BA75DE8D2}"/>
+              <c16:uniqueId val="{00000003-8E9B-40F0-9C5A-A1C094762365}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5502,7 +5502,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$86</c:f>
+              <c:f>Trend!$A$94</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5536,7 +5536,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -5574,7 +5574,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$86:$K$86</c:f>
+              <c:f>Trend!$B$94:$K$94</c:f>
               <c:numCache>
                 <c:formatCode>0.00"x"</c:formatCode>
                 <c:ptCount val="10"/>
@@ -5614,7 +5614,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-1FCD-4D7C-9E44-342BA75DE8D2}"/>
+              <c16:uniqueId val="{00000004-8E9B-40F0-9C5A-A1C094762365}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5691,7 +5691,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="2115092272"/>
+        <c:axId val="1142395951"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5726,12 +5726,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="64994688"/>
+        <c:crossAx val="1658445983"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="64994688"/>
+        <c:axId val="1658445983"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5741,7 +5741,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="2115092272"/>
+        <c:crossAx val="1142395951"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -5800,7 +5800,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$93</c:f>
+              <c:f>Trend!$A$101</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5821,7 +5821,7 @@
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -5859,7 +5859,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$93:$K$93</c:f>
+              <c:f>Trend!$B$101:$K$101</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -5911,7 +5911,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-81AF-428A-B852-FF523D478B10}"/>
+              <c16:uniqueId val="{00000000-0275-4D9B-8BB4-D6F559259ABF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5924,8 +5924,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="64988192"/>
-        <c:axId val="2115079792"/>
+        <c:axId val="1658442271"/>
+        <c:axId val="1142393071"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -5935,7 +5935,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$89</c:f>
+              <c:f>Trend!$A$97</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5969,7 +5969,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -6007,7 +6007,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$89:$K$89</c:f>
+              <c:f>Trend!$B$97:$K$97</c:f>
               <c:numCache>
                 <c:formatCode>0.0"x"</c:formatCode>
                 <c:ptCount val="10"/>
@@ -6047,7 +6047,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-81AF-428A-B852-FF523D478B10}"/>
+              <c16:uniqueId val="{00000001-0275-4D9B-8BB4-D6F559259ABF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6056,7 +6056,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$90</c:f>
+              <c:f>Trend!$A$98</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6090,7 +6090,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -6128,7 +6128,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$90:$K$90</c:f>
+              <c:f>Trend!$B$98:$K$98</c:f>
               <c:numCache>
                 <c:formatCode>0.0"x"</c:formatCode>
                 <c:ptCount val="10"/>
@@ -6168,7 +6168,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-81AF-428A-B852-FF523D478B10}"/>
+              <c16:uniqueId val="{00000002-0275-4D9B-8BB4-D6F559259ABF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6177,7 +6177,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$91</c:f>
+              <c:f>Trend!$A$99</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6211,7 +6211,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -6249,7 +6249,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$91:$K$91</c:f>
+              <c:f>Trend!$B$99:$K$99</c:f>
               <c:numCache>
                 <c:formatCode>0.0"x"</c:formatCode>
                 <c:ptCount val="10"/>
@@ -6289,7 +6289,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-81AF-428A-B852-FF523D478B10}"/>
+              <c16:uniqueId val="{00000003-0275-4D9B-8BB4-D6F559259ABF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6298,7 +6298,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$92</c:f>
+              <c:f>Trend!$A$100</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6332,7 +6332,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -6370,7 +6370,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$92:$K$92</c:f>
+              <c:f>Trend!$B$100:$K$100</c:f>
               <c:numCache>
                 <c:formatCode>0.0"x"</c:formatCode>
                 <c:ptCount val="10"/>
@@ -6410,7 +6410,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-81AF-428A-B852-FF523D478B10}"/>
+              <c16:uniqueId val="{00000004-0275-4D9B-8BB4-D6F559259ABF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6487,7 +6487,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="2115079792"/>
+        <c:axId val="1142393071"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -6522,12 +6522,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="64988192"/>
+        <c:crossAx val="1658442271"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="64988192"/>
+        <c:axId val="1658442271"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6537,7 +6537,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="2115079792"/>
+        <c:crossAx val="1142393071"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6596,7 +6596,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$100</c:f>
+              <c:f>Trend!$A$108</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6617,7 +6617,7 @@
           <c:invertIfNegative val="1"/>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -6655,7 +6655,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$100:$K$100</c:f>
+              <c:f>Trend!$B$108:$K$108</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -6707,7 +6707,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-EC5F-491D-8BD4-F4D190E9CAEE}"/>
+              <c16:uniqueId val="{00000000-D3C8-4C75-86B8-00BF8B6EBEBF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6720,8 +6720,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="64980304"/>
-        <c:axId val="2115085552"/>
+        <c:axId val="1658445055"/>
+        <c:axId val="1142415151"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -6731,7 +6731,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$95</c:f>
+              <c:f>Trend!$A$103</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6765,7 +6765,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -6803,7 +6803,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$95:$K$95</c:f>
+              <c:f>Trend!$B$103:$K$103</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -6843,7 +6843,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-EC5F-491D-8BD4-F4D190E9CAEE}"/>
+              <c16:uniqueId val="{00000001-D3C8-4C75-86B8-00BF8B6EBEBF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6852,7 +6852,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$96</c:f>
+              <c:f>Trend!$A$104</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6886,7 +6886,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -6924,7 +6924,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$96:$K$96</c:f>
+              <c:f>Trend!$B$104:$K$104</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -6964,7 +6964,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-EC5F-491D-8BD4-F4D190E9CAEE}"/>
+              <c16:uniqueId val="{00000002-D3C8-4C75-86B8-00BF8B6EBEBF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6973,7 +6973,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$97</c:f>
+              <c:f>Trend!$A$105</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7007,7 +7007,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -7045,7 +7045,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$97:$K$97</c:f>
+              <c:f>Trend!$B$105:$K$105</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -7085,7 +7085,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-EC5F-491D-8BD4-F4D190E9CAEE}"/>
+              <c16:uniqueId val="{00000003-D3C8-4C75-86B8-00BF8B6EBEBF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7094,7 +7094,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$98</c:f>
+              <c:f>Trend!$A$106</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7128,7 +7128,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -7166,7 +7166,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$98:$K$98</c:f>
+              <c:f>Trend!$B$106:$K$106</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -7206,7 +7206,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-EC5F-491D-8BD4-F4D190E9CAEE}"/>
+              <c16:uniqueId val="{00000004-D3C8-4C75-86B8-00BF8B6EBEBF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7215,7 +7215,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>Trend!$A$99</c:f>
+              <c:f>Trend!$A$107</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7249,7 +7249,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Trend!$B$62:$K$62</c:f>
+              <c:f>Trend!$B$70:$K$70</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -7287,7 +7287,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Trend!$B$99:$K$99</c:f>
+              <c:f>Trend!$B$107:$K$107</c:f>
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="10"/>
@@ -7327,7 +7327,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-EC5F-491D-8BD4-F4D190E9CAEE}"/>
+              <c16:uniqueId val="{00000005-D3C8-4C75-86B8-00BF8B6EBEBF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7404,7 +7404,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="2115085552"/>
+        <c:axId val="1142415151"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -7439,12 +7439,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="64980304"/>
+        <c:crossAx val="1658445055"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="64980304"/>
+        <c:axId val="1658445055"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7454,7 +7454,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="2115085552"/>
+        <c:crossAx val="1142415151"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -7486,7 +7486,7 @@
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6120000" cy="3420000"/>
+    <xdr:ext cx="5760000" cy="3600000"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -7512,12 +7512,12 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6120000" cy="3420000"/>
+    <xdr:ext cx="5760000" cy="3600000"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="3" name="Chart 2">
@@ -7545,10 +7545,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6120000" cy="3420000"/>
+    <xdr:ext cx="5760000" cy="3600000"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="4" name="Chart 3">
@@ -7574,12 +7574,12 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6120000" cy="3420000"/>
+    <xdr:ext cx="5760000" cy="3600000"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="5" name="Chart 4">
@@ -7607,10 +7607,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6120000" cy="3420000"/>
+    <xdr:ext cx="5760000" cy="3600000"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="6" name="Chart 5">
@@ -7636,12 +7636,12 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6120000" cy="3420000"/>
+    <xdr:ext cx="5760000" cy="3600000"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="7" name="Chart 6">
@@ -15332,11 +15332,11 @@
     <tabColor rgb="FF1F3864"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="11" width="9" customWidth="1"/>
+    <col min="2" max="23" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="25.8" x14ac:dyDescent="0.5">
@@ -15349,1527 +15349,1591 @@
         <v>218</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A61" s="46" t="s">
+    <row r="4" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="17" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="18" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="19" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="20" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="21" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="22" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="23" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="24" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="25" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="26" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="27" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="28" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="29" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="30" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="31" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="32" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="33" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="34" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="35" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="36" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="37" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="38" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="39" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="40" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="41" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="42" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="43" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="44" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="45" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="46" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="47" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="48" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="50" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="55" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="65" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="66" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="67" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" s="46" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A62" s="60" t="s">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70" s="60" t="s">
         <v>220</v>
       </c>
-      <c r="B62" s="19" t="s">
+      <c r="B70" s="19" t="s">
         <v>221</v>
       </c>
-      <c r="C62" s="19" t="s">
+      <c r="C70" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="D62" s="19" t="s">
+      <c r="D70" s="19" t="s">
         <v>223</v>
       </c>
-      <c r="E62" s="19" t="s">
+      <c r="E70" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="F62" s="19" t="s">
+      <c r="F70" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="G62" s="19" t="s">
+      <c r="G70" s="19" t="s">
         <v>226</v>
       </c>
-      <c r="H62" s="19" t="s">
+      <c r="H70" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="I62" s="19" t="s">
+      <c r="I70" s="19" t="s">
         <v>228</v>
       </c>
-      <c r="J62" s="19" t="s">
+      <c r="J70" s="19" t="s">
         <v>229</v>
       </c>
-      <c r="K62" s="19" t="s">
+      <c r="K70" s="19" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A63" s="12" t="s">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B63" s="61">
+      <c r="B71" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!B7),'Ratio Calculations'!B7,NA())</f>
         <v>0.24944267499381903</v>
       </c>
-      <c r="C63" s="61">
+      <c r="C71" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!C7),'Ratio Calculations'!C7,NA())</f>
         <v>0.24682256167790528</v>
       </c>
-      <c r="D63" s="61">
+      <c r="D71" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!D7),'Ratio Calculations'!D7,NA())</f>
         <v>0.24499489544979808</v>
       </c>
-      <c r="E63" s="61">
+      <c r="E71" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!E7),'Ratio Calculations'!E7,NA())</f>
         <v>0.24103622438577799</v>
       </c>
-      <c r="F63" s="61">
+      <c r="F71" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!F7),'Ratio Calculations'!F7,NA())</f>
         <v>0.24299348201565829</v>
       </c>
-      <c r="G63" s="61">
+      <c r="G71" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!G7),'Ratio Calculations'!G7,NA())</f>
         <v>0.24440170353070476</v>
       </c>
-      <c r="H63" s="61">
+      <c r="H71" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!H7),'Ratio Calculations'!H7,NA())</f>
         <v>0.23463353364769649</v>
       </c>
-      <c r="I63" s="61">
+      <c r="I71" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!I7),'Ratio Calculations'!I7,NA())</f>
         <v>0.23729570504032604</v>
       </c>
-      <c r="J63" s="61">
+      <c r="J71" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!J7),'Ratio Calculations'!J7,NA())</f>
         <v>0.24132813866676156</v>
       </c>
-      <c r="K63" s="61">
+      <c r="K71" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!K7),'Ratio Calculations'!K7,NA())</f>
         <v>0.24209350620670911</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A64" s="12" t="s">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="B64" s="61">
+      <c r="B72" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!B8),'Ratio Calculations'!B8,NA())</f>
         <v>0.13323899291604546</v>
       </c>
-      <c r="C64" s="61">
+      <c r="C72" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!C8),'Ratio Calculations'!C8,NA())</f>
         <v>0.13286572369695795</v>
       </c>
-      <c r="D64" s="61">
+      <c r="D72" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!D8),'Ratio Calculations'!D8,NA())</f>
         <v>0.13013505113861107</v>
       </c>
-      <c r="E64" s="61">
+      <c r="E72" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!E8),'Ratio Calculations'!E8,NA())</f>
         <v>0.12977479158890134</v>
       </c>
-      <c r="F64" s="61">
+      <c r="F72" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!F8),'Ratio Calculations'!F8,NA())</f>
         <v>0.13085793440912444</v>
       </c>
-      <c r="G64" s="61">
+      <c r="G72" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!G8),'Ratio Calculations'!G8,NA())</f>
         <v>0.12884769482822858</v>
       </c>
-      <c r="H64" s="61">
+      <c r="H72" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!H8),'Ratio Calculations'!H8,NA())</f>
         <v>0.12148717361227385</v>
       </c>
-      <c r="I64" s="61">
+      <c r="I72" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!I8),'Ratio Calculations'!I8,NA())</f>
         <v>0.12259688802674482</v>
       </c>
-      <c r="J64" s="61">
+      <c r="J72" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!J8),'Ratio Calculations'!J8,NA())</f>
         <v>0.1261333134213391</v>
       </c>
-      <c r="K64" s="61">
+      <c r="K72" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!K8),'Ratio Calculations'!K8,NA())</f>
         <v>0.12843206714262356</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="12" t="s">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="B65" s="61">
+      <c r="B73" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!B9),'Ratio Calculations'!B9,NA())</f>
         <v>0.22399576892064124</v>
       </c>
-      <c r="C65" s="61">
+      <c r="C73" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!C9),'Ratio Calculations'!C9,NA())</f>
         <v>0.22281797534068787</v>
       </c>
-      <c r="D65" s="61">
+      <c r="D73" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!D9),'Ratio Calculations'!D9,NA())</f>
         <v>0.21952040179890359</v>
       </c>
-      <c r="E65" s="61">
+      <c r="E73" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!E9),'Ratio Calculations'!E9,NA())</f>
         <v>0.22072845624192466</v>
       </c>
-      <c r="F65" s="61">
+      <c r="F73" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!F9),'Ratio Calculations'!F9,NA())</f>
         <v>0.23321861462059804</v>
       </c>
-      <c r="G65" s="61">
+      <c r="G73" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!G9),'Ratio Calculations'!G9,NA())</f>
         <v>0.22009892086330934</v>
       </c>
-      <c r="H65" s="61">
+      <c r="H73" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!H9),'Ratio Calculations'!H9,NA())</f>
         <v>0.21434256498806134</v>
       </c>
-      <c r="I65" s="61">
+      <c r="I73" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!I9),'Ratio Calculations'!I9,NA())</f>
         <v>0.22236885076546764</v>
       </c>
-      <c r="J65" s="61">
+      <c r="J73" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!J9),'Ratio Calculations'!J9,NA())</f>
         <v>0.22704131916831494</v>
       </c>
-      <c r="K65" s="61">
+      <c r="K73" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!K9),'Ratio Calculations'!K9,NA())</f>
         <v>0.23300957722057408</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A66" s="12" t="s">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="B66" s="61" t="e">
+      <c r="B74" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!B10),'Ratio Calculations'!B10,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="C66" s="61" t="e">
+      <c r="C74" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!C10),'Ratio Calculations'!C10,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="D66" s="61" t="e">
+      <c r="D74" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!D10),'Ratio Calculations'!D10,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E66" s="61" t="e">
+      <c r="E74" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!E10),'Ratio Calculations'!E10,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F66" s="61" t="e">
+      <c r="F74" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!F10),'Ratio Calculations'!F10,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="G66" s="61" t="e">
+      <c r="G74" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!G10),'Ratio Calculations'!G10,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="H66" s="61">
+      <c r="H74" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!H10),'Ratio Calculations'!H10,NA())</f>
         <v>0.10387100598731401</v>
       </c>
-      <c r="I66" s="61">
+      <c r="I74" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!I10),'Ratio Calculations'!I10,NA())</f>
         <v>0.1094350131702619</v>
       </c>
-      <c r="J66" s="61">
+      <c r="J74" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!J10),'Ratio Calculations'!J10,NA())</f>
         <v>0.11306766550677098</v>
       </c>
-      <c r="K66" s="61">
+      <c r="K74" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!K10),'Ratio Calculations'!K10,NA())</f>
         <v>0.11348707197763802</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="12" t="s">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A75" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B67" s="61">
+      <c r="B75" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!B11),'Ratio Calculations'!B11,NA())</f>
         <v>0.34412363266344442</v>
       </c>
-      <c r="C67" s="61">
+      <c r="C75" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!C11),'Ratio Calculations'!C11,NA())</f>
         <v>0.33668122270742357</v>
       </c>
-      <c r="D67" s="61" t="e">
+      <c r="D75" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!D11),'Ratio Calculations'!D11,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E67" s="61" t="e">
+      <c r="E75" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!E11),'Ratio Calculations'!E11,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F67" s="61" t="e">
+      <c r="F75" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!F11),'Ratio Calculations'!F11,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="G67" s="61" t="e">
+      <c r="G75" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!G11),'Ratio Calculations'!G11,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="H67" s="61" t="e">
+      <c r="H75" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!H11),'Ratio Calculations'!H11,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="I67" s="61" t="e">
+      <c r="I75" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!I11),'Ratio Calculations'!I11,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="J67" s="61" t="e">
+      <c r="J75" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!J11),'Ratio Calculations'!J11,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="K67" s="61" t="e">
+      <c r="K75" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!K11),'Ratio Calculations'!K11,NA())</f>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="13" t="s">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="B68" s="13" t="e">
-        <f t="shared" ref="B68:K68" si="0">IF(AND(B$62&gt;="FY2020",B$62&lt;="FY2023"),1,NA())</f>
+      <c r="B76" s="13" t="e">
+        <f t="shared" ref="B76:K76" si="0">IF(AND(B$70&gt;="FY2020",B$70&lt;="FY2023"),1,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="C68" s="13" t="e">
+      <c r="C76" s="13" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="D68" s="13" t="e">
+      <c r="D76" s="13" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="E68" s="13" t="e">
+      <c r="E76" s="13" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="F68" s="13">
+      <c r="F76" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G68" s="13">
+      <c r="G76" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H68" s="13">
+      <c r="H76" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="I68" s="13">
+      <c r="I76" s="13">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="J68" s="13" t="e">
+      <c r="J76" s="13" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="K68" s="13" t="e">
+      <c r="K76" s="13" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="12" t="s">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A78" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B70" s="62">
+      <c r="B78" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!B21),'Ratio Calculations'!B21,NA())</f>
         <v>2.8345144675961997E-2</v>
       </c>
-      <c r="C70" s="62">
+      <c r="C78" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!C21),'Ratio Calculations'!C21,NA())</f>
         <v>1.989264988573123E-2</v>
       </c>
-      <c r="D70" s="62">
+      <c r="D78" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!D21),'Ratio Calculations'!D21,NA())</f>
         <v>1.3069999941214393E-2</v>
       </c>
-      <c r="E70" s="62">
+      <c r="E78" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!E21),'Ratio Calculations'!E21,NA())</f>
         <v>2.8621380734950744E-2</v>
       </c>
-      <c r="F70" s="62">
+      <c r="F78" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!F21),'Ratio Calculations'!F21,NA())</f>
         <v>2.4332127233071522E-2</v>
       </c>
-      <c r="G70" s="62">
+      <c r="G78" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!G21),'Ratio Calculations'!G21,NA())</f>
         <v>2.4082273910547024E-2</v>
       </c>
-      <c r="H70" s="62">
+      <c r="H78" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!H21),'Ratio Calculations'!H21,NA())</f>
         <v>1.9277712950232801E-2</v>
       </c>
-      <c r="I70" s="62">
+      <c r="I78" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!I21),'Ratio Calculations'!I21,NA())</f>
         <v>2.4136487628318944E-2</v>
       </c>
-      <c r="J70" s="62">
+      <c r="J78" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!J21),'Ratio Calculations'!J21,NA())</f>
         <v>2.881379551633859E-2</v>
       </c>
-      <c r="K70" s="62">
+      <c r="K78" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!K21),'Ratio Calculations'!K21,NA())</f>
         <v>3.0991785258765055E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="12" t="s">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A79" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="B71" s="62">
+      <c r="B79" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!B22),'Ratio Calculations'!B22,NA())</f>
         <v>1.9794641127367986E-2</v>
       </c>
-      <c r="C71" s="62">
+      <c r="C79" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!C22),'Ratio Calculations'!C22,NA())</f>
         <v>2.0763417942259253E-2</v>
       </c>
-      <c r="D71" s="62">
+      <c r="D79" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!D22),'Ratio Calculations'!D22,NA())</f>
         <v>2.2136520314177545E-2</v>
       </c>
-      <c r="E71" s="62">
+      <c r="E79" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!E22),'Ratio Calculations'!E22,NA())</f>
         <v>2.3961546269555937E-2</v>
       </c>
-      <c r="F71" s="62">
+      <c r="F79" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!F22),'Ratio Calculations'!F22,NA())</f>
         <v>2.3998416896036844E-2</v>
       </c>
-      <c r="G71" s="62">
+      <c r="G79" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!G22),'Ratio Calculations'!G22,NA())</f>
         <v>2.5555175599324246E-2</v>
       </c>
-      <c r="H71" s="62">
+      <c r="H79" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!H22),'Ratio Calculations'!H22,NA())</f>
         <v>2.5749711395260715E-2</v>
       </c>
-      <c r="I71" s="62">
+      <c r="I79" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!I22),'Ratio Calculations'!I22,NA())</f>
         <v>2.5968880267448098E-2</v>
       </c>
-      <c r="J71" s="62">
+      <c r="J79" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!J22),'Ratio Calculations'!J22,NA())</f>
         <v>2.8952301603832536E-2</v>
       </c>
-      <c r="K71" s="62">
+      <c r="K79" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!K22),'Ratio Calculations'!K22,NA())</f>
         <v>2.9425763438516175E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A72" s="12" t="s">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A80" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="B72" s="62">
+      <c r="B80" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!B23),'Ratio Calculations'!B23,NA())</f>
         <v>1.7123733060509638E-2</v>
       </c>
-      <c r="C72" s="62">
+      <c r="C80" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!C23),'Ratio Calculations'!C23,NA())</f>
         <v>1.5468851395197923E-2</v>
       </c>
-      <c r="D72" s="62">
+      <c r="D80" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!D23),'Ratio Calculations'!D23,NA())</f>
         <v>2.552276532186587E-2</v>
       </c>
-      <c r="E72" s="62">
+      <c r="E80" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!E23),'Ratio Calculations'!E23,NA())</f>
         <v>1.3566557087483441E-2</v>
       </c>
-      <c r="F72" s="62">
+      <c r="F80" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!F23),'Ratio Calculations'!F23,NA())</f>
         <v>1.9509728448731303E-2</v>
       </c>
-      <c r="G72" s="62">
+      <c r="G80" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!G23),'Ratio Calculations'!G23,NA())</f>
         <v>1.2002494778370851E-2</v>
       </c>
-      <c r="H72" s="62">
+      <c r="H80" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!H23),'Ratio Calculations'!H23,NA())</f>
         <v>1.5135776821486868E-2</v>
       </c>
-      <c r="I72" s="62">
+      <c r="I80" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!I23),'Ratio Calculations'!I23,NA())</f>
         <v>1.4422916708322502E-2</v>
       </c>
-      <c r="J72" s="62">
+      <c r="J80" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!J23),'Ratio Calculations'!J23,NA())</f>
         <v>1.81140950089381E-2</v>
       </c>
-      <c r="K72" s="62">
+      <c r="K80" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!K23),'Ratio Calculations'!K23,NA())</f>
         <v>6.8815106812424648E-3</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A73" s="12" t="s">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A81" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B73" s="62">
+      <c r="B81" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!B25),'Ratio Calculations'!B25,NA())</f>
         <v>3.2243703892139403E-2</v>
       </c>
-      <c r="C73" s="62">
+      <c r="C81" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!C25),'Ratio Calculations'!C25,NA())</f>
         <v>1.5283842794759825E-2</v>
       </c>
-      <c r="D73" s="62" t="e">
+      <c r="D81" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!D25),'Ratio Calculations'!D25,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E73" s="62" t="e">
+      <c r="E81" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!E25),'Ratio Calculations'!E25,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F73" s="62" t="e">
+      <c r="F81" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!F25),'Ratio Calculations'!F25,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="G73" s="62" t="e">
+      <c r="G81" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!G25),'Ratio Calculations'!G25,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="H73" s="62" t="e">
+      <c r="H81" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!H25),'Ratio Calculations'!H25,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="I73" s="62" t="e">
+      <c r="I81" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!I25),'Ratio Calculations'!I25,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="J73" s="62" t="e">
+      <c r="J81" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!J25),'Ratio Calculations'!J25,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="K73" s="62" t="e">
+      <c r="K81" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!K25),'Ratio Calculations'!K25,NA())</f>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A74" s="13" t="s">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A82" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="B74" s="13" t="e">
-        <f t="shared" ref="B74:K74" si="1">IF(AND(B$62&gt;="FY2020",B$62&lt;="FY2023"),1,NA())</f>
+      <c r="B82" s="13" t="e">
+        <f t="shared" ref="B82:K82" si="1">IF(AND(B$70&gt;="FY2020",B$70&lt;="FY2023"),1,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="C74" s="13" t="e">
+      <c r="C82" s="13" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="D74" s="13" t="e">
+      <c r="D82" s="13" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="E74" s="13" t="e">
+      <c r="E82" s="13" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="F74" s="13">
+      <c r="F82" s="13">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="G74" s="13">
+      <c r="G82" s="13">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="H74" s="13">
+      <c r="H82" s="13">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="I74" s="13">
+      <c r="I82" s="13">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J74" s="13" t="e">
+      <c r="J82" s="13" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
-      <c r="K74" s="13" t="e">
+      <c r="K82" s="13" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A76" s="12" t="s">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A84" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B76" s="62">
+      <c r="B84" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!B14),'Ratio Calculations'!B14,NA())</f>
         <v>4.7295233702528687E-2</v>
       </c>
-      <c r="C76" s="62">
+      <c r="C84" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!C14),'Ratio Calculations'!C14,NA())</f>
         <v>4.1223492771718634E-2</v>
       </c>
-      <c r="D76" s="62">
+      <c r="D84" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!D14),'Ratio Calculations'!D14,NA())</f>
         <v>4.3025185713529902E-2</v>
       </c>
-      <c r="E76" s="62">
+      <c r="E84" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!E14),'Ratio Calculations'!E14,NA())</f>
         <v>3.9559475771552104E-2</v>
       </c>
-      <c r="F76" s="62">
+      <c r="F84" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!F14),'Ratio Calculations'!F14,NA())</f>
         <v>4.0609978153315816E-2</v>
       </c>
-      <c r="G76" s="62">
+      <c r="G84" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!G14),'Ratio Calculations'!G14,NA())</f>
         <v>4.5691680669012719E-2</v>
       </c>
-      <c r="H76" s="62">
+      <c r="H84" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!H14),'Ratio Calculations'!H14,NA())</f>
         <v>3.3716191793437988E-2</v>
       </c>
-      <c r="I76" s="62">
+      <c r="I84" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!I14),'Ratio Calculations'!I14,NA())</f>
         <v>4.2033060654770887E-2</v>
       </c>
-      <c r="J76" s="62">
+      <c r="J84" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!J14),'Ratio Calculations'!J14,NA())</f>
         <v>4.3508297531050885E-2</v>
       </c>
-      <c r="K76" s="62">
+      <c r="K84" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!K14),'Ratio Calculations'!K14,NA())</f>
         <v>4.222034418958881E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A77" s="12" t="s">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A85" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="B77" s="62">
+      <c r="B85" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!B15),'Ratio Calculations'!B15,NA())</f>
         <v>3.0930179667955426E-2</v>
       </c>
-      <c r="C77" s="62">
+      <c r="C85" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!C15),'Ratio Calculations'!C15,NA())</f>
         <v>3.1862042239875994E-2</v>
       </c>
-      <c r="D77" s="62">
+      <c r="D85" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!D15),'Ratio Calculations'!D15,NA())</f>
         <v>3.164378143188111E-2</v>
       </c>
-      <c r="E77" s="62">
+      <c r="E85" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!E15),'Ratio Calculations'!E15,NA())</f>
         <v>3.1021001552032378E-2</v>
       </c>
-      <c r="F77" s="62">
+      <c r="F85" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!F15),'Ratio Calculations'!F15,NA())</f>
         <v>3.259155318089961E-2</v>
       </c>
-      <c r="G77" s="62">
+      <c r="G85" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!G15),'Ratio Calculations'!G15,NA())</f>
         <v>3.4236891935343926E-2</v>
       </c>
-      <c r="H77" s="62">
+      <c r="H85" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!H15),'Ratio Calculations'!H15,NA())</f>
         <v>3.4337354706240032E-2</v>
       </c>
-      <c r="I77" s="62">
+      <c r="I85" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!I15),'Ratio Calculations'!I15,NA())</f>
         <v>3.3488794419910026E-2</v>
       </c>
-      <c r="J77" s="62">
+      <c r="J85" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!J15),'Ratio Calculations'!J15,NA())</f>
         <v>3.6490039417888566E-2</v>
       </c>
-      <c r="K77" s="62">
+      <c r="K85" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!K15),'Ratio Calculations'!K15,NA())</f>
         <v>3.7724126655403561E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A78" s="12" t="s">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A86" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="B78" s="62">
+      <c r="B86" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!B16),'Ratio Calculations'!B16,NA())</f>
         <v>2.9929684316394565E-2</v>
       </c>
-      <c r="C78" s="62">
+      <c r="C86" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!C16),'Ratio Calculations'!C16,NA())</f>
         <v>2.1187540558079171E-2</v>
       </c>
-      <c r="D78" s="62">
+      <c r="D86" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!D16),'Ratio Calculations'!D16,NA())</f>
         <v>2.1452253553491122E-2</v>
       </c>
-      <c r="E78" s="62">
+      <c r="E86" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!E16),'Ratio Calculations'!E16,NA())</f>
         <v>1.8407667271805438E-2</v>
       </c>
-      <c r="F78" s="62">
+      <c r="F86" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!F16),'Ratio Calculations'!F16,NA())</f>
         <v>2.0981448776585306E-2</v>
       </c>
-      <c r="G78" s="62">
+      <c r="G86" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!G16),'Ratio Calculations'!G16,NA())</f>
         <v>2.5216117428637736E-2</v>
       </c>
-      <c r="H78" s="62">
+      <c r="H86" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!H16),'Ratio Calculations'!H16,NA())</f>
         <v>2.7829864155728527E-2</v>
       </c>
-      <c r="I78" s="62">
+      <c r="I86" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!I16),'Ratio Calculations'!I16,NA())</f>
         <v>2.0634634994901327E-2</v>
       </c>
-      <c r="J78" s="62">
+      <c r="J86" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!J16),'Ratio Calculations'!J16,NA())</f>
         <v>2.6161782997899716E-2</v>
       </c>
-      <c r="K78" s="62">
+      <c r="K86" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!K16),'Ratio Calculations'!K16,NA())</f>
         <v>1.2801235420815215E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A79" s="12" t="s">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A87" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="B79" s="62">
+      <c r="B87" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!B17),'Ratio Calculations'!B17,NA())</f>
         <v>2.8379674017257911E-2</v>
       </c>
-      <c r="C79" s="62">
+      <c r="C87" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!C17),'Ratio Calculations'!C17,NA())</f>
         <v>1.5451904890570117E-2</v>
       </c>
-      <c r="D79" s="62">
+      <c r="D87" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!D17),'Ratio Calculations'!D17,NA())</f>
         <v>2.6279845778799771E-2</v>
       </c>
-      <c r="E79" s="62">
+      <c r="E87" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!E17),'Ratio Calculations'!E17,NA())</f>
         <v>2.7928969927881346E-2</v>
       </c>
-      <c r="F79" s="62">
+      <c r="F87" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!F17),'Ratio Calculations'!F17,NA())</f>
         <v>2.9823188859333438E-2</v>
       </c>
-      <c r="G79" s="62">
+      <c r="G87" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!G17),'Ratio Calculations'!G17,NA())</f>
         <v>3.0711294795801838E-2</v>
       </c>
-      <c r="H79" s="62">
+      <c r="H87" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!H17),'Ratio Calculations'!H17,NA())</f>
         <v>2.3285316260596361E-2</v>
       </c>
-      <c r="I79" s="62">
+      <c r="I87" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!I17),'Ratio Calculations'!I17,NA())</f>
         <v>2.5435430905441002E-2</v>
       </c>
-      <c r="J79" s="62">
+      <c r="J87" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!J17),'Ratio Calculations'!J17,NA())</f>
         <v>2.6640661362175581E-2</v>
       </c>
-      <c r="K79" s="62">
+      <c r="K87" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!K17),'Ratio Calculations'!K17,NA())</f>
         <v>2.6253830027414934E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A80" s="12" t="s">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A88" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B80" s="62">
+      <c r="B88" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!B18),'Ratio Calculations'!B18,NA())</f>
         <v>5.4502671076062069E-2</v>
       </c>
-      <c r="C80" s="62">
+      <c r="C88" s="62">
         <f>IF(ISNUMBER('Ratio Calculations'!C18),'Ratio Calculations'!C18,NA())</f>
         <v>2.8633811603243919E-2</v>
       </c>
-      <c r="D80" s="62" t="e">
+      <c r="D88" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!D18),'Ratio Calculations'!D18,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E80" s="62" t="e">
+      <c r="E88" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!E18),'Ratio Calculations'!E18,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F80" s="62" t="e">
+      <c r="F88" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!F18),'Ratio Calculations'!F18,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="G80" s="62" t="e">
+      <c r="G88" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!G18),'Ratio Calculations'!G18,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="H80" s="62" t="e">
+      <c r="H88" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!H18),'Ratio Calculations'!H18,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="I80" s="62" t="e">
+      <c r="I88" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!I18),'Ratio Calculations'!I18,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="J80" s="62" t="e">
+      <c r="J88" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!J18),'Ratio Calculations'!J18,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="K80" s="62" t="e">
+      <c r="K88" s="62" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!K18),'Ratio Calculations'!K18,NA())</f>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A81" s="13" t="s">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A89" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="B81" s="13" t="e">
-        <f t="shared" ref="B81:K81" si="2">IF(AND(B$62&gt;="FY2020",B$62&lt;="FY2023"),1,NA())</f>
+      <c r="B89" s="13" t="e">
+        <f t="shared" ref="B89:K89" si="2">IF(AND(B$70&gt;="FY2020",B$70&lt;="FY2023"),1,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="C81" s="13" t="e">
+      <c r="C89" s="13" t="e">
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="D81" s="13" t="e">
+      <c r="D89" s="13" t="e">
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="E81" s="13" t="e">
+      <c r="E89" s="13" t="e">
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="F81" s="13">
+      <c r="F89" s="13">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="G81" s="13">
+      <c r="G89" s="13">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="H81" s="13">
+      <c r="H89" s="13">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="I81" s="13">
+      <c r="I89" s="13">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="J81" s="13" t="e">
+      <c r="J89" s="13" t="e">
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="K81" s="13" t="e">
+      <c r="K89" s="13" t="e">
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A83" s="12" t="s">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A91" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B83" s="63">
+      <c r="B91" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!B28),'Ratio Calculations'!B28,NA())</f>
         <v>0.86195613196270615</v>
       </c>
-      <c r="C83" s="63">
+      <c r="C91" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!C28),'Ratio Calculations'!C28,NA())</f>
         <v>0.75984768405904157</v>
       </c>
-      <c r="D83" s="63">
+      <c r="D91" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!D28),'Ratio Calculations'!D28,NA())</f>
         <v>0.79890806303806294</v>
       </c>
-      <c r="E83" s="63">
+      <c r="E91" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!E28),'Ratio Calculations'!E28,NA())</f>
         <v>0.7945237177015041</v>
       </c>
-      <c r="F83" s="63">
+      <c r="F91" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!F28),'Ratio Calculations'!F28,NA())</f>
         <v>0.97217334988396564</v>
       </c>
-      <c r="G83" s="63">
+      <c r="G91" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!G28),'Ratio Calculations'!G28,NA())</f>
         <v>0.92779729683333523</v>
       </c>
-      <c r="H83" s="63">
+      <c r="H91" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!H28),'Ratio Calculations'!H28,NA())</f>
         <v>0.82057094513980777</v>
       </c>
-      <c r="I83" s="63">
+      <c r="I91" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!I28),'Ratio Calculations'!I28,NA())</f>
         <v>0.83186712113834338</v>
       </c>
-      <c r="J83" s="63">
+      <c r="J91" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!J28),'Ratio Calculations'!J28,NA())</f>
         <v>0.82268284602004471</v>
       </c>
-      <c r="K83" s="63">
+      <c r="K91" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!K28),'Ratio Calculations'!K28,NA())</f>
         <v>0.78975332421442468</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A84" s="12" t="s">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A92" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="B84" s="63">
+      <c r="B92" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!B29),'Ratio Calculations'!B29,NA())</f>
         <v>0.97707865168539321</v>
       </c>
-      <c r="C84" s="63">
+      <c r="C92" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!C29),'Ratio Calculations'!C29,NA())</f>
         <v>0.98982566447556442</v>
       </c>
-      <c r="D84" s="63">
+      <c r="D92" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!D29),'Ratio Calculations'!D29,NA())</f>
         <v>1.0182174043962662</v>
       </c>
-      <c r="E84" s="63">
+      <c r="E92" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!E29),'Ratio Calculations'!E29,NA())</f>
         <v>1.0106726341610364</v>
       </c>
-      <c r="F84" s="63">
+      <c r="F92" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!F29),'Ratio Calculations'!F29,NA())</f>
         <v>1.1318628240218966</v>
       </c>
-      <c r="G84" s="63">
+      <c r="G92" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!G29),'Ratio Calculations'!G29,NA())</f>
         <v>1.0021738392038313</v>
       </c>
-      <c r="H84" s="63">
+      <c r="H92" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!H29),'Ratio Calculations'!H29,NA())</f>
         <v>1.0218138633664604</v>
       </c>
-      <c r="I84" s="63">
+      <c r="I92" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!I29),'Ratio Calculations'!I29,NA())</f>
         <v>1.0683679242473871</v>
       </c>
-      <c r="J84" s="63">
+      <c r="J92" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!J29),'Ratio Calculations'!J29,NA())</f>
         <v>0.96565531242950597</v>
       </c>
-      <c r="K84" s="63">
+      <c r="K92" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!K29),'Ratio Calculations'!K29,NA())</f>
         <v>1.0342783227336423</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A85" s="12" t="s">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A93" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="B85" s="63">
+      <c r="B93" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!B30),'Ratio Calculations'!B30,NA())</f>
         <v>0.80404354587869364</v>
       </c>
-      <c r="C85" s="63">
+      <c r="C93" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!C30),'Ratio Calculations'!C30,NA())</f>
         <v>0.78305275762485027</v>
       </c>
-      <c r="D85" s="63">
+      <c r="D93" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!D30),'Ratio Calculations'!D30,NA())</f>
         <v>0.75683060109289613</v>
       </c>
-      <c r="E85" s="63">
+      <c r="E93" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!E30),'Ratio Calculations'!E30,NA())</f>
         <v>0.76458611247630415</v>
       </c>
-      <c r="F85" s="63">
+      <c r="F93" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!F30),'Ratio Calculations'!F30,NA())</f>
         <v>0.81367955225823241</v>
       </c>
-      <c r="G85" s="63">
+      <c r="G93" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!G30),'Ratio Calculations'!G30,NA())</f>
         <v>0.74581878331189122</v>
       </c>
-      <c r="H85" s="63">
+      <c r="H93" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!H30),'Ratio Calculations'!H30,NA())</f>
         <v>0.73500406079591596</v>
       </c>
-      <c r="I85" s="63">
+      <c r="I93" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!I30),'Ratio Calculations'!I30,NA())</f>
         <v>0.80632706439158053</v>
       </c>
-      <c r="J85" s="63">
+      <c r="J93" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!J30),'Ratio Calculations'!J30,NA())</f>
         <v>0.95815558343789209</v>
       </c>
-      <c r="K85" s="63">
+      <c r="K93" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!K30),'Ratio Calculations'!K30,NA())</f>
         <v>0.80102717031146453</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A86" s="12" t="s">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A94" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B86" s="63">
+      <c r="B94" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!B32),'Ratio Calculations'!B32,NA())</f>
         <v>1.4727815063385534</v>
       </c>
-      <c r="C86" s="63">
+      <c r="C94" s="63">
         <f>IF(ISNUMBER('Ratio Calculations'!C32),'Ratio Calculations'!C32,NA())</f>
         <v>1.5830258302583027</v>
       </c>
-      <c r="D86" s="63" t="e">
+      <c r="D94" s="63" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!D32),'Ratio Calculations'!D32,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E86" s="63" t="e">
+      <c r="E94" s="63" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!E32),'Ratio Calculations'!E32,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F86" s="63" t="e">
+      <c r="F94" s="63" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!F32),'Ratio Calculations'!F32,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="G86" s="63" t="e">
+      <c r="G94" s="63" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!G32),'Ratio Calculations'!G32,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="H86" s="63" t="e">
+      <c r="H94" s="63" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!H32),'Ratio Calculations'!H32,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="I86" s="63" t="e">
+      <c r="I94" s="63" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!I32),'Ratio Calculations'!I32,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="J86" s="63" t="e">
+      <c r="J94" s="63" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!J32),'Ratio Calculations'!J32,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="K86" s="63" t="e">
+      <c r="K94" s="63" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!K32),'Ratio Calculations'!K32,NA())</f>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A87" s="13" t="s">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A95" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="B87" s="13" t="e">
-        <f t="shared" ref="B87:K87" si="3">IF(AND(B$62&gt;="FY2020",B$62&lt;="FY2023"),1,NA())</f>
+      <c r="B95" s="13" t="e">
+        <f t="shared" ref="B95:K95" si="3">IF(AND(B$70&gt;="FY2020",B$70&lt;="FY2023"),1,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="C87" s="13" t="e">
+      <c r="C95" s="13" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
-      <c r="D87" s="13" t="e">
+      <c r="D95" s="13" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
-      <c r="E87" s="13" t="e">
+      <c r="E95" s="13" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
-      <c r="F87" s="13">
+      <c r="F95" s="13">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="G87" s="13">
+      <c r="G95" s="13">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="H87" s="13">
+      <c r="H95" s="13">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="I87" s="13">
+      <c r="I95" s="13">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="J87" s="13" t="e">
+      <c r="J95" s="13" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
-      <c r="K87" s="13" t="e">
+      <c r="K95" s="13" t="e">
         <f t="shared" si="3"/>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A89" s="12" t="s">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A97" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B89" s="64">
+      <c r="B97" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!B35),'Ratio Calculations'!B35,NA())</f>
         <v>0.57041038057987214</v>
       </c>
-      <c r="C89" s="64">
+      <c r="C97" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!C35),'Ratio Calculations'!C35,NA())</f>
         <v>0.57517755066689757</v>
       </c>
-      <c r="D89" s="64">
+      <c r="D97" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!D35),'Ratio Calculations'!D35,NA())</f>
         <v>0.72874651530753198</v>
       </c>
-      <c r="E89" s="64">
+      <c r="E97" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!E35),'Ratio Calculations'!E35,NA())</f>
         <v>0.66790514027859527</v>
       </c>
-      <c r="F89" s="64">
+      <c r="F97" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!F35),'Ratio Calculations'!F35,NA())</f>
         <v>0.55832790668448895</v>
       </c>
-      <c r="G89" s="64">
+      <c r="G97" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!G35),'Ratio Calculations'!G35,NA())</f>
         <v>0.46610658279918599</v>
       </c>
-      <c r="H89" s="64">
+      <c r="H97" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!H35),'Ratio Calculations'!H35,NA())</f>
         <v>0.53277455405114982</v>
       </c>
-      <c r="I89" s="64">
+      <c r="I97" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!I35),'Ratio Calculations'!I35,NA())</f>
         <v>0.51899855006696261</v>
       </c>
-      <c r="J89" s="64">
+      <c r="J97" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!J35),'Ratio Calculations'!J35,NA())</f>
         <v>0.47002186386918632</v>
       </c>
-      <c r="K89" s="64">
+      <c r="K97" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!K35),'Ratio Calculations'!K35,NA())</f>
         <v>0.48658475544684426</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A90" s="12" t="s">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A98" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="B90" s="64">
+      <c r="B98" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!B36),'Ratio Calculations'!B36,NA())</f>
         <v>0.44883230619526437</v>
       </c>
-      <c r="C90" s="64">
+      <c r="C98" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!C36),'Ratio Calculations'!C36,NA())</f>
         <v>0.63534615037458253</v>
       </c>
-      <c r="D90" s="64">
+      <c r="D98" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!D36),'Ratio Calculations'!D36,NA())</f>
         <v>0.53224452415477375</v>
       </c>
-      <c r="E90" s="64">
+      <c r="E98" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!E36),'Ratio Calculations'!E36,NA())</f>
         <v>0.46483572895277209</v>
       </c>
-      <c r="F90" s="64">
+      <c r="F98" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!F36),'Ratio Calculations'!F36,NA())</f>
         <v>0.44357123763699546</v>
       </c>
-      <c r="G90" s="64">
+      <c r="G98" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!G36),'Ratio Calculations'!G36,NA())</f>
         <v>0.47256333665228456</v>
       </c>
-      <c r="H90" s="64">
+      <c r="H98" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!H36),'Ratio Calculations'!H36,NA())</f>
         <v>0.39642563084225313</v>
       </c>
-      <c r="I90" s="64">
+      <c r="I98" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!I36),'Ratio Calculations'!I36,NA())</f>
         <v>0.31486950275361164</v>
       </c>
-      <c r="J90" s="64">
+      <c r="J98" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!J36),'Ratio Calculations'!J36,NA())</f>
         <v>0.31305562611125221</v>
       </c>
-      <c r="K90" s="64">
+      <c r="K98" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!K36),'Ratio Calculations'!K36,NA())</f>
         <v>0.24917706761761074</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A91" s="12" t="s">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A99" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="B91" s="64">
+      <c r="B99" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!B37),'Ratio Calculations'!B37,NA())</f>
         <v>2.0979135618479883</v>
       </c>
-      <c r="C91" s="64">
+      <c r="C99" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!C37),'Ratio Calculations'!C37,NA())</f>
         <v>2.2576393917451121</v>
       </c>
-      <c r="D91" s="64">
+      <c r="D99" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!D37),'Ratio Calculations'!D37,NA())</f>
         <v>1.9437141033822591</v>
       </c>
-      <c r="E91" s="64">
+      <c r="E99" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!E37),'Ratio Calculations'!E37,NA())</f>
         <v>1.6418989851860493</v>
       </c>
-      <c r="F91" s="64">
+      <c r="F99" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!F37),'Ratio Calculations'!F37,NA())</f>
         <v>1.4045026178010471</v>
       </c>
-      <c r="G91" s="64">
+      <c r="G99" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!G37),'Ratio Calculations'!G37,NA())</f>
         <v>1.4173295153250609</v>
       </c>
-      <c r="H91" s="64">
+      <c r="H99" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!H37),'Ratio Calculations'!H37,NA())</f>
         <v>1.3359296984222089</v>
       </c>
-      <c r="I91" s="64">
+      <c r="I99" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!I37),'Ratio Calculations'!I37,NA())</f>
         <v>1.053874665977071</v>
       </c>
-      <c r="J91" s="64">
+      <c r="J99" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!J37),'Ratio Calculations'!J37,NA())</f>
         <v>2.1621784808597995</v>
       </c>
-      <c r="K91" s="64">
+      <c r="K99" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!K37),'Ratio Calculations'!K37,NA())</f>
         <v>2.9592318059299192</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A92" s="12" t="s">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A100" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B92" s="64">
+      <c r="B100" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!B39),'Ratio Calculations'!B39,NA())</f>
         <v>0.32599255583126552</v>
       </c>
-      <c r="C92" s="64">
+      <c r="C100" s="64">
         <f>IF(ISNUMBER('Ratio Calculations'!C39),'Ratio Calculations'!C39,NA())</f>
         <v>0.31574344023323614</v>
       </c>
-      <c r="D92" s="64" t="e">
+      <c r="D100" s="64" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!D39),'Ratio Calculations'!D39,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E92" s="64" t="e">
+      <c r="E100" s="64" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!E39),'Ratio Calculations'!E39,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F92" s="64" t="e">
+      <c r="F100" s="64" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!F39),'Ratio Calculations'!F39,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="G92" s="64" t="e">
+      <c r="G100" s="64" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!G39),'Ratio Calculations'!G39,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="H92" s="64" t="e">
+      <c r="H100" s="64" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!H39),'Ratio Calculations'!H39,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="I92" s="64" t="e">
+      <c r="I100" s="64" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!I39),'Ratio Calculations'!I39,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="J92" s="64" t="e">
+      <c r="J100" s="64" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!J39),'Ratio Calculations'!J39,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="K92" s="64" t="e">
+      <c r="K100" s="64" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!K39),'Ratio Calculations'!K39,NA())</f>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A93" s="13" t="s">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A101" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="B93" s="13" t="e">
-        <f t="shared" ref="B93:K93" si="4">IF(AND(B$62&gt;="FY2020",B$62&lt;="FY2023"),1,NA())</f>
+      <c r="B101" s="13" t="e">
+        <f t="shared" ref="B101:K101" si="4">IF(AND(B$70&gt;="FY2020",B$70&lt;="FY2023"),1,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="C93" s="13" t="e">
+      <c r="C101" s="13" t="e">
         <f t="shared" si="4"/>
         <v>#N/A</v>
       </c>
-      <c r="D93" s="13" t="e">
+      <c r="D101" s="13" t="e">
         <f t="shared" si="4"/>
         <v>#N/A</v>
       </c>
-      <c r="E93" s="13" t="e">
+      <c r="E101" s="13" t="e">
         <f t="shared" si="4"/>
         <v>#N/A</v>
       </c>
-      <c r="F93" s="13">
+      <c r="F101" s="13">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="G93" s="13">
+      <c r="G101" s="13">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="H93" s="13">
+      <c r="H101" s="13">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="I93" s="13">
+      <c r="I101" s="13">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="J93" s="13" t="e">
+      <c r="J101" s="13" t="e">
         <f t="shared" si="4"/>
         <v>#N/A</v>
       </c>
-      <c r="K93" s="13" t="e">
+      <c r="K101" s="13" t="e">
         <f t="shared" si="4"/>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A95" s="12" t="s">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A103" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B95" s="61">
+      <c r="B103" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!B49),'Ratio Calculations'!B49,NA())</f>
         <v>5.6475573217666941E-3</v>
       </c>
-      <c r="C95" s="61">
+      <c r="C103" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!C49),'Ratio Calculations'!C49,NA())</f>
         <v>3.000932857139893E-2</v>
       </c>
-      <c r="D95" s="61">
+      <c r="D103" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!D49),'Ratio Calculations'!D49,NA())</f>
         <v>2.9385127107618425E-2</v>
       </c>
-      <c r="E95" s="61">
+      <c r="E103" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!E49),'Ratio Calculations'!E49,NA())</f>
         <v>1.8805515657546401E-2</v>
       </c>
-      <c r="F95" s="61">
+      <c r="F103" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!F49),'Ratio Calculations'!F49,NA())</f>
         <v>6.7907740716948162E-2</v>
       </c>
-      <c r="G95" s="61">
+      <c r="G103" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!G49),'Ratio Calculations'!G49,NA())</f>
         <v>2.2565301414001038E-2</v>
       </c>
-      <c r="H95" s="61">
+      <c r="H103" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!H49),'Ratio Calculations'!H49,NA())</f>
         <v>6.7139047699564358E-2</v>
       </c>
-      <c r="I95" s="61">
+      <c r="I103" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!I49),'Ratio Calculations'!I49,NA())</f>
         <v>6.0665378184824981E-2</v>
       </c>
-      <c r="J95" s="61">
+      <c r="J103" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!J49),'Ratio Calculations'!J49,NA())</f>
         <v>4.9640776986074497E-2</v>
       </c>
-      <c r="K95" s="61">
+      <c r="K103" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!K49),'Ratio Calculations'!K49,NA())</f>
         <v>4.7254565346948496E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A96" s="12" t="s">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A104" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="B96" s="61">
+      <c r="B104" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!B50),'Ratio Calculations'!B50,NA())</f>
         <v>2.1686933622492521E-2</v>
       </c>
-      <c r="C96" s="61">
+      <c r="C104" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!C50),'Ratio Calculations'!C50,NA())</f>
         <v>8.6810030407937999E-2</v>
       </c>
-      <c r="D96" s="61">
+      <c r="D104" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!D50),'Ratio Calculations'!D50,NA())</f>
         <v>9.7275721759348954E-2</v>
       </c>
-      <c r="E96" s="61">
+      <c r="E104" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!E50),'Ratio Calculations'!E50,NA())</f>
         <v>7.8593829462620723E-2</v>
       </c>
-      <c r="F96" s="61">
+      <c r="F104" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!F50),'Ratio Calculations'!F50,NA())</f>
         <v>9.2061059704131587E-2</v>
       </c>
-      <c r="G96" s="61">
+      <c r="G104" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!G50),'Ratio Calculations'!G50,NA())</f>
         <v>0.17490900150514799</v>
       </c>
-      <c r="H96" s="61">
+      <c r="H104" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!H50),'Ratio Calculations'!H50,NA())</f>
         <v>0.15834817714580285</v>
       </c>
-      <c r="I96" s="61">
+      <c r="I104" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!I50),'Ratio Calculations'!I50,NA())</f>
         <v>6.7573164606043568E-2</v>
       </c>
-      <c r="J96" s="61">
+      <c r="J104" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!J50),'Ratio Calculations'!J50,NA())</f>
         <v>5.0200173345990251E-2</v>
       </c>
-      <c r="K96" s="61">
+      <c r="K104" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!K50),'Ratio Calculations'!K50,NA())</f>
         <v>8.1673236314761422E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A97" s="12" t="s">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A105" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="B97" s="61">
+      <c r="B105" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!B51),'Ratio Calculations'!B51,NA())</f>
         <v>5.0141127196576596E-2</v>
       </c>
-      <c r="C97" s="61">
+      <c r="C105" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!C51),'Ratio Calculations'!C51,NA())</f>
         <v>6.8867752759305345E-2</v>
       </c>
-      <c r="D97" s="61">
+      <c r="D105" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!D51),'Ratio Calculations'!D51,NA())</f>
         <v>-1.158338741077225E-2</v>
       </c>
-      <c r="E97" s="61">
+      <c r="E105" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!E51),'Ratio Calculations'!E51,NA())</f>
         <v>3.5616977973278452E-3</v>
       </c>
-      <c r="F97" s="61">
+      <c r="F105" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!F51),'Ratio Calculations'!F51,NA())</f>
         <v>8.3509150679554445E-2</v>
       </c>
-      <c r="G97" s="61">
+      <c r="G105" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!G51),'Ratio Calculations'!G51,NA())</f>
         <v>4.0679859318631273E-2</v>
       </c>
-      <c r="H97" s="61">
+      <c r="H105" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!H51),'Ratio Calculations'!H51,NA())</f>
         <v>7.5205964260849356E-2</v>
       </c>
-      <c r="I97" s="61">
+      <c r="I105" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!I51),'Ratio Calculations'!I51,NA())</f>
         <v>1.2012842477303165E-2</v>
       </c>
-      <c r="J97" s="61">
+      <c r="J105" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!J51),'Ratio Calculations'!J51,NA())</f>
         <v>-1.9434946913802431E-2</v>
       </c>
-      <c r="K97" s="61">
+      <c r="K105" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!K51),'Ratio Calculations'!K51,NA())</f>
         <v>3.5276605289451535E-3</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A98" s="12" t="s">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A106" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="B98" s="61">
+      <c r="B106" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!B52),'Ratio Calculations'!B52,NA())</f>
         <v>9.4495671148024929E-3</v>
       </c>
-      <c r="C98" s="61">
+      <c r="C106" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!C52),'Ratio Calculations'!C52,NA())</f>
         <v>3.226706179726313E-2</v>
       </c>
-      <c r="D98" s="61">
+      <c r="D106" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!D52),'Ratio Calculations'!D52,NA())</f>
         <v>-2.3253850310726798E-2</v>
       </c>
-      <c r="E98" s="61">
+      <c r="E106" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!E52),'Ratio Calculations'!E52,NA())</f>
         <v>1.6476771728418438E-2</v>
       </c>
-      <c r="F98" s="61">
+      <c r="F106" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!F52),'Ratio Calculations'!F52,NA())</f>
         <v>8.7052660225880985E-2</v>
       </c>
-      <c r="G98" s="61">
+      <c r="G106" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!G52),'Ratio Calculations'!G52,NA())</f>
         <v>0.15093099671412924</v>
       </c>
-      <c r="H98" s="61">
+      <c r="H106" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!H52),'Ratio Calculations'!H52,NA())</f>
         <v>0.14667736146609389</v>
       </c>
-      <c r="I98" s="61">
+      <c r="I106" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!I52),'Ratio Calculations'!I52,NA())</f>
         <v>2.1744027506076291E-2</v>
       </c>
-      <c r="J98" s="61">
+      <c r="J106" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!J52),'Ratio Calculations'!J52,NA())</f>
         <v>4.7099641443971274E-2</v>
       </c>
-      <c r="K98" s="61">
+      <c r="K106" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!K52),'Ratio Calculations'!K52,NA())</f>
         <v>3.077417495955137E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A99" s="12" t="s">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A107" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B99" s="61">
+      <c r="B107" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!B53),'Ratio Calculations'!B53,NA())</f>
         <v>2.1768795893170489E-2</v>
       </c>
-      <c r="C99" s="61">
+      <c r="C107" s="61">
         <f>IF(ISNUMBER('Ratio Calculations'!C53),'Ratio Calculations'!C53,NA())</f>
         <v>1.9460697023658158E-2</v>
       </c>
-      <c r="D99" s="61" t="e">
+      <c r="D107" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!D53),'Ratio Calculations'!D53,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E99" s="61" t="e">
+      <c r="E107" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!E53),'Ratio Calculations'!E53,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F99" s="61" t="e">
+      <c r="F107" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!F53),'Ratio Calculations'!F53,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="G99" s="61" t="e">
+      <c r="G107" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!G53),'Ratio Calculations'!G53,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="H99" s="61" t="e">
+      <c r="H107" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!H53),'Ratio Calculations'!H53,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="I99" s="61" t="e">
+      <c r="I107" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!I53),'Ratio Calculations'!I53,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="J99" s="61" t="e">
+      <c r="J107" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!J53),'Ratio Calculations'!J53,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="K99" s="61" t="e">
+      <c r="K107" s="61" t="e">
         <f>IF(ISNUMBER('Ratio Calculations'!K53),'Ratio Calculations'!K53,NA())</f>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A100" s="13" t="s">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A108" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="B100" s="13" t="e">
-        <f t="shared" ref="B100:K100" si="5">IF(AND(B$62&gt;="FY2020",B$62&lt;="FY2023"),1,NA())</f>
+      <c r="B108" s="13" t="e">
+        <f t="shared" ref="B108:K108" si="5">IF(AND(B$70&gt;="FY2020",B$70&lt;="FY2023"),1,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="C100" s="13" t="e">
+      <c r="C108" s="13" t="e">
         <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
-      <c r="D100" s="13" t="e">
+      <c r="D108" s="13" t="e">
         <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
-      <c r="E100" s="13" t="e">
+      <c r="E108" s="13" t="e">
         <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
-      <c r="F100" s="13">
+      <c r="F108" s="13">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G100" s="13">
+      <c r="G108" s="13">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="H100" s="13">
+      <c r="H108" s="13">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="I100" s="13">
+      <c r="I108" s="13">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="J100" s="13" t="e">
+      <c r="J108" s="13" t="e">
         <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>
-      <c r="K100" s="13" t="e">
+      <c r="K108" s="13" t="e">
         <f t="shared" si="5"/>
         <v>#N/A</v>
       </c>

</xml_diff>

<commit_message>
Final workbook build: 948 live formulas, 0 errors, 18 tests passing
</commit_message>
<xml_diff>
--- a/output/Competitor_Scorecard.xlsx
+++ b/output/Competitor_Scorecard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Claude_Projects\competitor-scorecard\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED14B9D2-3388-4803-82BE-5A669939EE86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB08E1D-E0C2-4712-BE80-01B4D323DB08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2630,7 +2630,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-ACAF-4267-837E-CCCC41256D22}"/>
+              <c16:uniqueId val="{00000000-A59F-4B67-960A-4C631C53A183}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2643,8 +2643,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="2046334991"/>
-        <c:axId val="303940431"/>
+        <c:axId val="2059561904"/>
+        <c:axId val="67779984"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2766,7 +2766,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-ACAF-4267-837E-CCCC41256D22}"/>
+              <c16:uniqueId val="{00000001-A59F-4B67-960A-4C631C53A183}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2887,7 +2887,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-ACAF-4267-837E-CCCC41256D22}"/>
+              <c16:uniqueId val="{00000002-A59F-4B67-960A-4C631C53A183}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3008,7 +3008,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-ACAF-4267-837E-CCCC41256D22}"/>
+              <c16:uniqueId val="{00000003-A59F-4B67-960A-4C631C53A183}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3129,7 +3129,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-ACAF-4267-837E-CCCC41256D22}"/>
+              <c16:uniqueId val="{00000004-A59F-4B67-960A-4C631C53A183}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3250,7 +3250,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-ACAF-4267-837E-CCCC41256D22}"/>
+              <c16:uniqueId val="{00000005-A59F-4B67-960A-4C631C53A183}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3327,7 +3327,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="303940431"/>
+        <c:axId val="67779984"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -3362,12 +3362,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="2046334991"/>
+        <c:crossAx val="2059561904"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="2046334991"/>
+        <c:axId val="2059561904"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3377,7 +3377,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="303940431"/>
+        <c:crossAx val="67779984"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -3547,7 +3547,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2511-437A-9A64-B771344BDBB7}"/>
+              <c16:uniqueId val="{00000000-9185-40B0-82B4-1CDFAEF9060E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3560,8 +3560,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="907016159"/>
-        <c:axId val="303948111"/>
+        <c:axId val="659546656"/>
+        <c:axId val="67774224"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -3683,7 +3683,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-2511-437A-9A64-B771344BDBB7}"/>
+              <c16:uniqueId val="{00000001-9185-40B0-82B4-1CDFAEF9060E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3804,7 +3804,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-2511-437A-9A64-B771344BDBB7}"/>
+              <c16:uniqueId val="{00000002-9185-40B0-82B4-1CDFAEF9060E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3925,7 +3925,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-2511-437A-9A64-B771344BDBB7}"/>
+              <c16:uniqueId val="{00000003-9185-40B0-82B4-1CDFAEF9060E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4046,7 +4046,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-2511-437A-9A64-B771344BDBB7}"/>
+              <c16:uniqueId val="{00000004-9185-40B0-82B4-1CDFAEF9060E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4123,7 +4123,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="303948111"/>
+        <c:axId val="67774224"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4158,12 +4158,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="907016159"/>
+        <c:crossAx val="659546656"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="907016159"/>
+        <c:axId val="659546656"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4173,7 +4173,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="303948111"/>
+        <c:crossAx val="67774224"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -4343,7 +4343,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4561-4C80-8F29-AB00807C6161}"/>
+              <c16:uniqueId val="{00000000-2DF8-48AB-A24D-5791618528D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4356,8 +4356,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="907010127"/>
-        <c:axId val="303938031"/>
+        <c:axId val="659547584"/>
+        <c:axId val="67778064"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -4479,7 +4479,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4561-4C80-8F29-AB00807C6161}"/>
+              <c16:uniqueId val="{00000001-2DF8-48AB-A24D-5791618528D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4600,7 +4600,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-4561-4C80-8F29-AB00807C6161}"/>
+              <c16:uniqueId val="{00000002-2DF8-48AB-A24D-5791618528D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4721,7 +4721,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-4561-4C80-8F29-AB00807C6161}"/>
+              <c16:uniqueId val="{00000003-2DF8-48AB-A24D-5791618528D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4842,7 +4842,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-4561-4C80-8F29-AB00807C6161}"/>
+              <c16:uniqueId val="{00000004-2DF8-48AB-A24D-5791618528D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4963,7 +4963,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-4561-4C80-8F29-AB00807C6161}"/>
+              <c16:uniqueId val="{00000005-2DF8-48AB-A24D-5791618528D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5040,7 +5040,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="303938031"/>
+        <c:axId val="67778064"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5075,12 +5075,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="907010127"/>
+        <c:crossAx val="659547584"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="907010127"/>
+        <c:axId val="659547584"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5090,7 +5090,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="303938031"/>
+        <c:crossAx val="67778064"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -5260,7 +5260,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6DB2-4863-AF96-8ACF84C23459}"/>
+              <c16:uniqueId val="{00000000-EC1A-4A79-BF5E-5E2286822051}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5273,8 +5273,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="907011519"/>
-        <c:axId val="303936591"/>
+        <c:axId val="659547120"/>
+        <c:axId val="67776144"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -5396,7 +5396,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-6DB2-4863-AF96-8ACF84C23459}"/>
+              <c16:uniqueId val="{00000001-EC1A-4A79-BF5E-5E2286822051}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5517,7 +5517,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-6DB2-4863-AF96-8ACF84C23459}"/>
+              <c16:uniqueId val="{00000002-EC1A-4A79-BF5E-5E2286822051}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5638,7 +5638,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-6DB2-4863-AF96-8ACF84C23459}"/>
+              <c16:uniqueId val="{00000003-EC1A-4A79-BF5E-5E2286822051}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5759,7 +5759,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-6DB2-4863-AF96-8ACF84C23459}"/>
+              <c16:uniqueId val="{00000004-EC1A-4A79-BF5E-5E2286822051}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5836,7 +5836,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="303936591"/>
+        <c:axId val="67776144"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5871,12 +5871,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="907011519"/>
+        <c:crossAx val="659547120"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="907011519"/>
+        <c:axId val="659547120"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5886,7 +5886,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="303936591"/>
+        <c:crossAx val="67776144"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6056,7 +6056,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E72B-4CE9-ABE3-0984688A01D0}"/>
+              <c16:uniqueId val="{00000000-4512-4A56-B9A9-4C5548242D89}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6069,8 +6069,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="907012911"/>
-        <c:axId val="303947631"/>
+        <c:axId val="659549904"/>
+        <c:axId val="67780944"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -6192,7 +6192,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-E72B-4CE9-ABE3-0984688A01D0}"/>
+              <c16:uniqueId val="{00000001-4512-4A56-B9A9-4C5548242D89}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6313,7 +6313,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-E72B-4CE9-ABE3-0984688A01D0}"/>
+              <c16:uniqueId val="{00000002-4512-4A56-B9A9-4C5548242D89}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6434,7 +6434,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-E72B-4CE9-ABE3-0984688A01D0}"/>
+              <c16:uniqueId val="{00000003-4512-4A56-B9A9-4C5548242D89}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6555,7 +6555,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-E72B-4CE9-ABE3-0984688A01D0}"/>
+              <c16:uniqueId val="{00000004-4512-4A56-B9A9-4C5548242D89}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6632,7 +6632,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="303947631"/>
+        <c:axId val="67780944"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -6667,12 +6667,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="907012911"/>
+        <c:crossAx val="659549904"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="907012911"/>
+        <c:axId val="659549904"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6682,7 +6682,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="303947631"/>
+        <c:crossAx val="67780944"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6852,7 +6852,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-12D2-4A45-A779-E6BD3BA9E9AF}"/>
+              <c16:uniqueId val="{00000000-FA8D-43BF-BE65-C3588C728AA0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6865,8 +6865,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="907014767"/>
-        <c:axId val="303941391"/>
+        <c:axId val="659550832"/>
+        <c:axId val="2059448560"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -6988,7 +6988,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-12D2-4A45-A779-E6BD3BA9E9AF}"/>
+              <c16:uniqueId val="{00000001-FA8D-43BF-BE65-C3588C728AA0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7109,7 +7109,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-12D2-4A45-A779-E6BD3BA9E9AF}"/>
+              <c16:uniqueId val="{00000002-FA8D-43BF-BE65-C3588C728AA0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7230,7 +7230,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-12D2-4A45-A779-E6BD3BA9E9AF}"/>
+              <c16:uniqueId val="{00000003-FA8D-43BF-BE65-C3588C728AA0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7351,7 +7351,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-12D2-4A45-A779-E6BD3BA9E9AF}"/>
+              <c16:uniqueId val="{00000004-FA8D-43BF-BE65-C3588C728AA0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7472,7 +7472,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-12D2-4A45-A779-E6BD3BA9E9AF}"/>
+              <c16:uniqueId val="{00000005-FA8D-43BF-BE65-C3588C728AA0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7549,7 +7549,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="303941391"/>
+        <c:axId val="2059448560"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -7584,12 +7584,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="907014767"/>
+        <c:crossAx val="659550832"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="907014767"/>
+        <c:axId val="659550832"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7599,7 +7599,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="303941391"/>
+        <c:crossAx val="2059448560"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>

</xml_diff>

<commit_message>
Cover tagline: Accounting & financial analysis · SEC 10-K filings
</commit_message>
<xml_diff>
--- a/output/Competitor_Scorecard.xlsx
+++ b/output/Competitor_Scorecard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Claude_Projects\competitor-scorecard\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369FBDF0-4697-4798-891F-A4DFCED7CA32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7341E32-BE22-458E-96E1-E9C98334AAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -158,7 +158,7 @@
     <t>RYAN BARRY</t>
   </si>
   <si>
-    <t>Financial analysis · SEC filings</t>
+    <t>Accounting &amp; financial analysis · SEC 10-K filings</t>
   </si>
   <si>
     <t>01   —   COVER          ·          COMPETITOR SCORECARD   ·   FY2016–FY2025   ·   SEC 10-K DATA</t>
@@ -2667,7 +2667,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-326B-4322-9546-F87E005901F4}"/>
+              <c16:uniqueId val="{00000000-779D-4ADA-A6BF-1B88B886A6F2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2680,8 +2680,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="637261375"/>
-        <c:axId val="976272495"/>
+        <c:axId val="1521473887"/>
+        <c:axId val="974753423"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2803,7 +2803,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-326B-4322-9546-F87E005901F4}"/>
+              <c16:uniqueId val="{00000001-779D-4ADA-A6BF-1B88B886A6F2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2924,7 +2924,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-326B-4322-9546-F87E005901F4}"/>
+              <c16:uniqueId val="{00000002-779D-4ADA-A6BF-1B88B886A6F2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3045,7 +3045,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-326B-4322-9546-F87E005901F4}"/>
+              <c16:uniqueId val="{00000003-779D-4ADA-A6BF-1B88B886A6F2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3166,7 +3166,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-326B-4322-9546-F87E005901F4}"/>
+              <c16:uniqueId val="{00000004-779D-4ADA-A6BF-1B88B886A6F2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3287,7 +3287,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-326B-4322-9546-F87E005901F4}"/>
+              <c16:uniqueId val="{00000005-779D-4ADA-A6BF-1B88B886A6F2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3364,7 +3364,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="976272495"/>
+        <c:axId val="974753423"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -3399,12 +3399,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="637261375"/>
+        <c:crossAx val="1521473887"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="637261375"/>
+        <c:axId val="1521473887"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3414,7 +3414,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="976272495"/>
+        <c:crossAx val="974753423"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -3584,7 +3584,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B88F-416E-9BC4-522F8DC05362}"/>
+              <c16:uniqueId val="{00000000-1ED2-4F07-9980-BA7EC047A7F3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3597,8 +3597,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1523575135"/>
-        <c:axId val="976273455"/>
+        <c:axId val="1521471567"/>
+        <c:axId val="974752943"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -3720,7 +3720,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B88F-416E-9BC4-522F8DC05362}"/>
+              <c16:uniqueId val="{00000001-1ED2-4F07-9980-BA7EC047A7F3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3841,7 +3841,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-B88F-416E-9BC4-522F8DC05362}"/>
+              <c16:uniqueId val="{00000002-1ED2-4F07-9980-BA7EC047A7F3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3962,7 +3962,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-B88F-416E-9BC4-522F8DC05362}"/>
+              <c16:uniqueId val="{00000003-1ED2-4F07-9980-BA7EC047A7F3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4083,7 +4083,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-B88F-416E-9BC4-522F8DC05362}"/>
+              <c16:uniqueId val="{00000004-1ED2-4F07-9980-BA7EC047A7F3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4160,7 +4160,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="976273455"/>
+        <c:axId val="974752943"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4195,12 +4195,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1523575135"/>
+        <c:crossAx val="1521471567"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1523575135"/>
+        <c:axId val="1521471567"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4210,7 +4210,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="976273455"/>
+        <c:crossAx val="974752943"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -4380,7 +4380,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-AB87-4688-8413-B426E7B87831}"/>
+              <c16:uniqueId val="{00000000-33B7-4963-8C36-CE572A32F4AE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4393,8 +4393,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1523579311"/>
-        <c:axId val="976270575"/>
+        <c:axId val="1521475743"/>
+        <c:axId val="974756783"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -4516,7 +4516,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-AB87-4688-8413-B426E7B87831}"/>
+              <c16:uniqueId val="{00000001-33B7-4963-8C36-CE572A32F4AE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4637,7 +4637,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-AB87-4688-8413-B426E7B87831}"/>
+              <c16:uniqueId val="{00000002-33B7-4963-8C36-CE572A32F4AE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4758,7 +4758,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-AB87-4688-8413-B426E7B87831}"/>
+              <c16:uniqueId val="{00000003-33B7-4963-8C36-CE572A32F4AE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4879,7 +4879,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-AB87-4688-8413-B426E7B87831}"/>
+              <c16:uniqueId val="{00000004-33B7-4963-8C36-CE572A32F4AE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5000,7 +5000,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-AB87-4688-8413-B426E7B87831}"/>
+              <c16:uniqueId val="{00000005-33B7-4963-8C36-CE572A32F4AE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5077,7 +5077,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="976270575"/>
+        <c:axId val="974756783"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5112,12 +5112,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1523579311"/>
+        <c:crossAx val="1521475743"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1523579311"/>
+        <c:axId val="1521475743"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5127,7 +5127,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="976270575"/>
+        <c:crossAx val="974756783"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -5297,7 +5297,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-303F-4FBD-9022-A10A16313156}"/>
+              <c16:uniqueId val="{00000000-45C6-458E-8A04-AC6F9B8031B0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5310,8 +5310,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1523578847"/>
-        <c:axId val="976284975"/>
+        <c:axId val="1521474815"/>
+        <c:axId val="974748623"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -5433,7 +5433,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-303F-4FBD-9022-A10A16313156}"/>
+              <c16:uniqueId val="{00000001-45C6-458E-8A04-AC6F9B8031B0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5554,7 +5554,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-303F-4FBD-9022-A10A16313156}"/>
+              <c16:uniqueId val="{00000002-45C6-458E-8A04-AC6F9B8031B0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5675,7 +5675,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-303F-4FBD-9022-A10A16313156}"/>
+              <c16:uniqueId val="{00000003-45C6-458E-8A04-AC6F9B8031B0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5796,7 +5796,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-303F-4FBD-9022-A10A16313156}"/>
+              <c16:uniqueId val="{00000004-45C6-458E-8A04-AC6F9B8031B0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5873,7 +5873,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="976284975"/>
+        <c:axId val="974748623"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5908,12 +5908,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1523578847"/>
+        <c:crossAx val="1521474815"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1523578847"/>
+        <c:axId val="1521474815"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5923,7 +5923,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="976284975"/>
+        <c:crossAx val="974748623"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6093,7 +6093,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-47B6-47D0-900D-6B63ACBEFB4D}"/>
+              <c16:uniqueId val="{00000000-7ED8-492A-A692-2012C3DD8F4A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6106,8 +6106,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1523579775"/>
-        <c:axId val="976292175"/>
+        <c:axId val="1521473423"/>
+        <c:axId val="974756303"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -6229,7 +6229,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-47B6-47D0-900D-6B63ACBEFB4D}"/>
+              <c16:uniqueId val="{00000001-7ED8-492A-A692-2012C3DD8F4A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6350,7 +6350,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-47B6-47D0-900D-6B63ACBEFB4D}"/>
+              <c16:uniqueId val="{00000002-7ED8-492A-A692-2012C3DD8F4A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6471,7 +6471,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-47B6-47D0-900D-6B63ACBEFB4D}"/>
+              <c16:uniqueId val="{00000003-7ED8-492A-A692-2012C3DD8F4A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6592,7 +6592,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-47B6-47D0-900D-6B63ACBEFB4D}"/>
+              <c16:uniqueId val="{00000004-7ED8-492A-A692-2012C3DD8F4A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6669,7 +6669,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="976292175"/>
+        <c:axId val="974756303"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -6704,12 +6704,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1523579775"/>
+        <c:crossAx val="1521473423"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1523579775"/>
+        <c:axId val="1521473423"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6719,7 +6719,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="976292175"/>
+        <c:crossAx val="974756303"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6889,7 +6889,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5E12-4AA2-BF68-96CDDF9A4AEF}"/>
+              <c16:uniqueId val="{00000000-E860-440C-AC5F-8D44CB483B30}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6902,8 +6902,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1523574671"/>
-        <c:axId val="976285455"/>
+        <c:axId val="1521476671"/>
+        <c:axId val="974748143"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -7025,7 +7025,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-5E12-4AA2-BF68-96CDDF9A4AEF}"/>
+              <c16:uniqueId val="{00000001-E860-440C-AC5F-8D44CB483B30}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7146,7 +7146,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-5E12-4AA2-BF68-96CDDF9A4AEF}"/>
+              <c16:uniqueId val="{00000002-E860-440C-AC5F-8D44CB483B30}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7267,7 +7267,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-5E12-4AA2-BF68-96CDDF9A4AEF}"/>
+              <c16:uniqueId val="{00000003-E860-440C-AC5F-8D44CB483B30}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7388,7 +7388,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-5E12-4AA2-BF68-96CDDF9A4AEF}"/>
+              <c16:uniqueId val="{00000004-E860-440C-AC5F-8D44CB483B30}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7509,7 +7509,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-5E12-4AA2-BF68-96CDDF9A4AEF}"/>
+              <c16:uniqueId val="{00000005-E860-440C-AC5F-8D44CB483B30}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7586,7 +7586,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="976285455"/>
+        <c:axId val="974748143"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -7621,12 +7621,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1523574671"/>
+        <c:crossAx val="1521476671"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1523574671"/>
+        <c:axId val="1521476671"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7636,7 +7636,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="976285455"/>
+        <c:crossAx val="974748143"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>

</xml_diff>

<commit_message>
Cover band: tagline no longer clipped
</commit_message>
<xml_diff>
--- a/output/Competitor_Scorecard.xlsx
+++ b/output/Competitor_Scorecard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Claude_Projects\competitor-scorecard\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7341E32-BE22-458E-96E1-E9C98334AAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FC2C3B1-50E1-4CE5-BE00-EEA50953D4CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -158,10 +158,10 @@
     <t>RYAN BARRY</t>
   </si>
   <si>
+    <t>01   —   COVER          ·          COMPETITOR SCORECARD   ·   FY2016–FY2025   ·   SEC 10-K DATA</t>
+  </si>
+  <si>
     <t>Accounting &amp; financial analysis · SEC 10-K filings</t>
-  </si>
-  <si>
-    <t>01   —   COVER          ·          COMPETITOR SCORECARD   ·   FY2016–FY2025   ·   SEC 10-K DATA</t>
   </si>
   <si>
     <t>Competitor Scorecard:</t>
@@ -2230,11 +2230,11 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2667,7 +2667,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-779D-4ADA-A6BF-1B88B886A6F2}"/>
+              <c16:uniqueId val="{00000000-CC6D-4959-8027-CB23CDE9AD13}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2680,8 +2680,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1521473887"/>
-        <c:axId val="974753423"/>
+        <c:axId val="1006009728"/>
+        <c:axId val="1410632528"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2803,7 +2803,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-779D-4ADA-A6BF-1B88B886A6F2}"/>
+              <c16:uniqueId val="{00000001-CC6D-4959-8027-CB23CDE9AD13}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2924,7 +2924,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-779D-4ADA-A6BF-1B88B886A6F2}"/>
+              <c16:uniqueId val="{00000002-CC6D-4959-8027-CB23CDE9AD13}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3045,7 +3045,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-779D-4ADA-A6BF-1B88B886A6F2}"/>
+              <c16:uniqueId val="{00000003-CC6D-4959-8027-CB23CDE9AD13}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3166,7 +3166,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-779D-4ADA-A6BF-1B88B886A6F2}"/>
+              <c16:uniqueId val="{00000004-CC6D-4959-8027-CB23CDE9AD13}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3287,7 +3287,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-779D-4ADA-A6BF-1B88B886A6F2}"/>
+              <c16:uniqueId val="{00000005-CC6D-4959-8027-CB23CDE9AD13}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3364,7 +3364,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="974753423"/>
+        <c:axId val="1410632528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -3399,12 +3399,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1521473887"/>
+        <c:crossAx val="1006009728"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1521473887"/>
+        <c:axId val="1006009728"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3414,7 +3414,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="974753423"/>
+        <c:crossAx val="1410632528"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -3584,7 +3584,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1ED2-4F07-9980-BA7EC047A7F3}"/>
+              <c16:uniqueId val="{00000000-B8FA-4744-B7CA-64D0E646FB3C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3597,8 +3597,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1521471567"/>
-        <c:axId val="974752943"/>
+        <c:axId val="1006006016"/>
+        <c:axId val="1410645968"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -3720,7 +3720,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-1ED2-4F07-9980-BA7EC047A7F3}"/>
+              <c16:uniqueId val="{00000001-B8FA-4744-B7CA-64D0E646FB3C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3841,7 +3841,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-1ED2-4F07-9980-BA7EC047A7F3}"/>
+              <c16:uniqueId val="{00000002-B8FA-4744-B7CA-64D0E646FB3C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3962,7 +3962,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-1ED2-4F07-9980-BA7EC047A7F3}"/>
+              <c16:uniqueId val="{00000003-B8FA-4744-B7CA-64D0E646FB3C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4083,7 +4083,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-1ED2-4F07-9980-BA7EC047A7F3}"/>
+              <c16:uniqueId val="{00000004-B8FA-4744-B7CA-64D0E646FB3C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4160,7 +4160,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="974752943"/>
+        <c:axId val="1410645968"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4195,12 +4195,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1521471567"/>
+        <c:crossAx val="1006006016"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1521471567"/>
+        <c:axId val="1006006016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4210,7 +4210,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="974752943"/>
+        <c:crossAx val="1410645968"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -4380,7 +4380,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-33B7-4963-8C36-CE572A32F4AE}"/>
+              <c16:uniqueId val="{00000000-EB25-40D0-9AAF-2D3C8FF3942E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4393,8 +4393,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1521475743"/>
-        <c:axId val="974756783"/>
+        <c:axId val="1005993024"/>
+        <c:axId val="1410645008"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -4516,7 +4516,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-33B7-4963-8C36-CE572A32F4AE}"/>
+              <c16:uniqueId val="{00000001-EB25-40D0-9AAF-2D3C8FF3942E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4637,7 +4637,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-33B7-4963-8C36-CE572A32F4AE}"/>
+              <c16:uniqueId val="{00000002-EB25-40D0-9AAF-2D3C8FF3942E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4758,7 +4758,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-33B7-4963-8C36-CE572A32F4AE}"/>
+              <c16:uniqueId val="{00000003-EB25-40D0-9AAF-2D3C8FF3942E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4879,7 +4879,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-33B7-4963-8C36-CE572A32F4AE}"/>
+              <c16:uniqueId val="{00000004-EB25-40D0-9AAF-2D3C8FF3942E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5000,7 +5000,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-33B7-4963-8C36-CE572A32F4AE}"/>
+              <c16:uniqueId val="{00000005-EB25-40D0-9AAF-2D3C8FF3942E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5077,7 +5077,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="974756783"/>
+        <c:axId val="1410645008"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5112,12 +5112,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1521475743"/>
+        <c:crossAx val="1005993024"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1521475743"/>
+        <c:axId val="1005993024"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5127,7 +5127,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="974756783"/>
+        <c:crossAx val="1410645008"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -5297,7 +5297,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-45C6-458E-8A04-AC6F9B8031B0}"/>
+              <c16:uniqueId val="{00000000-30D7-4DB8-BEDE-F9F2FAF38E5D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5310,8 +5310,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1521474815"/>
-        <c:axId val="974748623"/>
+        <c:axId val="1005998128"/>
+        <c:axId val="1410651248"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -5433,7 +5433,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-45C6-458E-8A04-AC6F9B8031B0}"/>
+              <c16:uniqueId val="{00000001-30D7-4DB8-BEDE-F9F2FAF38E5D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5554,7 +5554,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-45C6-458E-8A04-AC6F9B8031B0}"/>
+              <c16:uniqueId val="{00000002-30D7-4DB8-BEDE-F9F2FAF38E5D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5675,7 +5675,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-45C6-458E-8A04-AC6F9B8031B0}"/>
+              <c16:uniqueId val="{00000003-30D7-4DB8-BEDE-F9F2FAF38E5D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5796,7 +5796,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-45C6-458E-8A04-AC6F9B8031B0}"/>
+              <c16:uniqueId val="{00000004-30D7-4DB8-BEDE-F9F2FAF38E5D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5873,7 +5873,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="974748623"/>
+        <c:axId val="1410651248"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5908,12 +5908,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1521474815"/>
+        <c:crossAx val="1005998128"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1521474815"/>
+        <c:axId val="1005998128"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5923,7 +5923,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="974748623"/>
+        <c:crossAx val="1410651248"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6093,7 +6093,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7ED8-492A-A692-2012C3DD8F4A}"/>
+              <c16:uniqueId val="{00000000-564F-4E61-BE28-9CCA807F7D17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6106,8 +6106,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1521473423"/>
-        <c:axId val="974756303"/>
+        <c:axId val="1005997200"/>
+        <c:axId val="1068119472"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -6229,7 +6229,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-7ED8-492A-A692-2012C3DD8F4A}"/>
+              <c16:uniqueId val="{00000001-564F-4E61-BE28-9CCA807F7D17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6350,7 +6350,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-7ED8-492A-A692-2012C3DD8F4A}"/>
+              <c16:uniqueId val="{00000002-564F-4E61-BE28-9CCA807F7D17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6471,7 +6471,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-7ED8-492A-A692-2012C3DD8F4A}"/>
+              <c16:uniqueId val="{00000003-564F-4E61-BE28-9CCA807F7D17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6592,7 +6592,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-7ED8-492A-A692-2012C3DD8F4A}"/>
+              <c16:uniqueId val="{00000004-564F-4E61-BE28-9CCA807F7D17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6669,7 +6669,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="974756303"/>
+        <c:axId val="1068119472"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -6704,12 +6704,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1521473423"/>
+        <c:crossAx val="1005997200"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1521473423"/>
+        <c:axId val="1005997200"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6719,7 +6719,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="974756303"/>
+        <c:crossAx val="1068119472"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6889,7 +6889,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E860-440C-AC5F-8D44CB483B30}"/>
+              <c16:uniqueId val="{00000000-016B-450D-9A73-9F7156A6B2C6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6902,8 +6902,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1521476671"/>
-        <c:axId val="974748143"/>
+        <c:axId val="1005994880"/>
+        <c:axId val="1410643088"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -7025,7 +7025,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-E860-440C-AC5F-8D44CB483B30}"/>
+              <c16:uniqueId val="{00000001-016B-450D-9A73-9F7156A6B2C6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7146,7 +7146,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-E860-440C-AC5F-8D44CB483B30}"/>
+              <c16:uniqueId val="{00000002-016B-450D-9A73-9F7156A6B2C6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7267,7 +7267,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-E860-440C-AC5F-8D44CB483B30}"/>
+              <c16:uniqueId val="{00000003-016B-450D-9A73-9F7156A6B2C6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7388,7 +7388,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-E860-440C-AC5F-8D44CB483B30}"/>
+              <c16:uniqueId val="{00000004-016B-450D-9A73-9F7156A6B2C6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7509,7 +7509,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-E860-440C-AC5F-8D44CB483B30}"/>
+              <c16:uniqueId val="{00000005-016B-450D-9A73-9F7156A6B2C6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7586,7 +7586,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="974748143"/>
+        <c:axId val="1410643088"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -7621,12 +7621,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1521476671"/>
+        <c:crossAx val="1005994880"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1521476671"/>
+        <c:axId val="1005994880"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7636,7 +7636,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="974748143"/>
+        <c:crossAx val="1410643088"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -8164,18 +8164,18 @@
       <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1"/>
+      <c r="D2" s="3" t="s">
+        <v>2</v>
+      </c>
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="83"/>
-      <c r="C3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="D3" s="1"/>
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>